<commit_message>
0.4.3 - Fixed bugs in Trainees Page and import trainees modal.
</commit_message>
<xml_diff>
--- a/keel_vessel_import_template.xlsx
+++ b/keel_vessel_import_template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF35E44-F3EE-4A3C-80B1-577FA58F6FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8EA0D37-994B-43A7-9CBC-131640DEB7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vessels" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
   <si>
     <t>Vessel Name</t>
   </si>
@@ -46,6 +46,21 @@
     <t>Vessel Type</t>
   </si>
   <si>
+    <t>Master Email (Optional)</t>
+  </si>
+  <si>
+    <t>CTO Deck Email (Optional)</t>
+  </si>
+  <si>
+    <t>CTO Engine Email (Optional)</t>
+  </si>
+  <si>
+    <t>CTO ETO Email (Optional)</t>
+  </si>
+  <si>
+    <t>CTO Catering Email (Optional)</t>
+  </si>
+  <si>
     <t>ABS (American Bureau of Shipping)</t>
   </si>
   <si>
@@ -118,61 +133,61 @@
     <t>Platform Support Vessel</t>
   </si>
   <si>
+    <t>Ocean Pioneer</t>
+  </si>
+  <si>
     <t>Singapore</t>
   </si>
   <si>
+    <t>Global Trader</t>
+  </si>
+  <si>
     <t>Panama</t>
   </si>
   <si>
+    <t>Energy Star</t>
+  </si>
+  <si>
     <t>Marshall Islands</t>
   </si>
   <si>
+    <t>Pacific Horizon</t>
+  </si>
+  <si>
     <t>Liberia</t>
   </si>
   <si>
+    <t>Chemical Explorer</t>
+  </si>
+  <si>
     <t>Hong Kong</t>
   </si>
   <si>
+    <t>Atlantic Bridge</t>
+  </si>
+  <si>
+    <t>Auto Prestige</t>
+  </si>
+  <si>
     <t>Japan</t>
   </si>
   <si>
+    <t>Deep Diver</t>
+  </si>
+  <si>
     <t>Norway</t>
   </si>
   <si>
+    <t>India Victory</t>
+  </si>
+  <si>
     <t>India</t>
   </si>
   <si>
+    <t>Nordic Spirit</t>
+  </si>
+  <si>
     <t>Bahamas</t>
-  </si>
-  <si>
-    <t>Ocean Pioneer</t>
-  </si>
-  <si>
-    <t>Global Trader</t>
-  </si>
-  <si>
-    <t>Energy Star</t>
-  </si>
-  <si>
-    <t>Pacific Horizon</t>
-  </si>
-  <si>
-    <t>Chemical Explorer</t>
-  </si>
-  <si>
-    <t>Atlantic Bridge</t>
-  </si>
-  <si>
-    <t>Auto Prestige</t>
-  </si>
-  <si>
-    <t>Deep Diver</t>
-  </si>
-  <si>
-    <t>India Victory</t>
-  </si>
-  <si>
-    <t>Nordic Spirit</t>
   </si>
 </sst>
 </file>
@@ -561,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -569,9 +584,10 @@
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="10" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,76 +603,171 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B2">
         <v>9123456</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F2" t="str">
+        <f>"master."&amp;LOWER(LEFT(A2,2)&amp;MID(A2,FIND(" ",A2,1)+1,2))&amp;"@keel.com"</f>
+        <v>master.ocpi@keel.com</v>
+      </c>
+      <c r="G2" t="str">
+        <f>"ctodeck."&amp;LOWER(LEFT(A2,2)&amp;MID(A2,FIND(" ",A2,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctodeck.ocpi@keel.com</v>
+      </c>
+      <c r="H2" t="str">
+        <f>"ctoeng."&amp;LOWER(LEFT(A2,2)&amp;MID(A2,FIND(" ",A2,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctoeng.ocpi@keel.com</v>
+      </c>
+      <c r="I2" t="str">
+        <f>"ctoeto."&amp;LOWER(LEFT(A2,2)&amp;MID(A2,FIND(" ",A2,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctoeto.ocpi@keel.com</v>
+      </c>
+      <c r="J2" t="str">
+        <f>"ctocat."&amp;LOWER(LEFT(A2,2)&amp;MID(A2,FIND(" ",A2,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctocat.ocpi@keel.com</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B3">
         <v>9234567</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F11" si="0">"master."&amp;LOWER(LEFT(A3,2)&amp;MID(A3,FIND(" ",A3,1)+1,2))&amp;"@keel.com"</f>
+        <v>master.gltr@keel.com</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" ref="G3:G11" si="1">"ctodeck."&amp;LOWER(LEFT(A3,2)&amp;MID(A3,FIND(" ",A3,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctodeck.gltr@keel.com</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H11" si="2">"ctoeng."&amp;LOWER(LEFT(A3,2)&amp;MID(A3,FIND(" ",A3,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctoeng.gltr@keel.com</v>
+      </c>
+      <c r="I3" t="str">
+        <f t="shared" ref="I3:I11" si="3">"ctoeto."&amp;LOWER(LEFT(A3,2)&amp;MID(A3,FIND(" ",A3,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctoeto.gltr@keel.com</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J11" si="4">"ctocat."&amp;LOWER(LEFT(A3,2)&amp;MID(A3,FIND(" ",A3,1)+1,2))&amp;"@keel.com"</f>
+        <v>ctocat.gltr@keel.com</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>9345678</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="0"/>
+        <v>master.enst@keel.com</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.enst@keel.com</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.enst@keel.com</v>
+      </c>
+      <c r="I4" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.enst@keel.com</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.enst@keel.com</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>9456789</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" t="str">
+        <f t="shared" si="0"/>
+        <v>master.paho@keel.com</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.paho@keel.com</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.paho@keel.com</v>
+      </c>
+      <c r="I5" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.paho@keel.com</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.paho@keel.com</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -664,98 +775,218 @@
         <v>9567890</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="0"/>
+        <v>master.chex@keel.com</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.chex@keel.com</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.chex@keel.com</v>
+      </c>
+      <c r="I6" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.chex@keel.com</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.chex@keel.com</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7">
         <v>9678901</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="0"/>
+        <v>master.atbr@keel.com</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.atbr@keel.com</v>
+      </c>
+      <c r="H7" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.atbr@keel.com</v>
+      </c>
+      <c r="I7" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.atbr@keel.com</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.atbr@keel.com</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8">
         <v>9789012</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>master.aupr@keel.com</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.aupr@keel.com</v>
+      </c>
+      <c r="H8" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.aupr@keel.com</v>
+      </c>
+      <c r="I8" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.aupr@keel.com</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.aupr@keel.com</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9">
         <v>9890123</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>master.dedi@keel.com</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.dedi@keel.com</v>
+      </c>
+      <c r="H9" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.dedi@keel.com</v>
+      </c>
+      <c r="I9" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.dedi@keel.com</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.dedi@keel.com</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B10">
         <v>9112233</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>master.invi@keel.com</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.invi@keel.com</v>
+      </c>
+      <c r="H10" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.invi@keel.com</v>
+      </c>
+      <c r="I10" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.invi@keel.com</v>
+      </c>
+      <c r="J10" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.invi@keel.com</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B11">
         <v>9223344</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>master.nosp@keel.com</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="1"/>
+        <v>ctodeck.nosp@keel.com</v>
+      </c>
+      <c r="H11" t="str">
+        <f t="shared" si="2"/>
+        <v>ctoeng.nosp@keel.com</v>
+      </c>
+      <c r="I11" t="str">
+        <f t="shared" si="3"/>
+        <v>ctoeto.nosp@keel.com</v>
+      </c>
+      <c r="J11" t="str">
+        <f t="shared" si="4"/>
+        <v>ctocat.nosp@keel.com</v>
       </c>
     </row>
   </sheetData>
@@ -764,17 +995,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Class" error="Please select a valid Classification Society from the list." xr:uid="{00000000-0002-0000-0000-000000000000}">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Selection" error="Please select a valid Classification Society from the provided list." xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
-            <xm:f>Reference!$A$1:$A$12</xm:f>
+            <xm:f>Reference!$A$1:$A$13</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D999</xm:sqref>
+          <xm:sqref>D2:D1000</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Type" error="Please select a valid Vessel Type from the list." xr:uid="{00000000-0002-0000-0000-000002000000}">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Selection" error="Please select a valid Vessel Type from the provided list." xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Reference!$B$1:$B$12</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E999</xm:sqref>
+          <xm:sqref>E2:E1000</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -784,103 +1015,108 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>